<commit_message>
Atualização automática - 18/08/2026 09:04
</commit_message>
<xml_diff>
--- a/dados/pesquisa/RESPOSTAS_PESQUISA_2.xlsx
+++ b/dados/pesquisa/RESPOSTAS_PESQUISA_2.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="235">
   <si>
     <t>Timestamp</t>
   </si>
@@ -645,6 +645,78 @@
   </si>
   <si>
     <t xml:space="preserve">Tudo último </t>
+  </si>
+  <si>
+    <t>Transporte, Alimentação e refeitório, Uniforme e equipamentos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bônus por ficar até o fim da temporada, Pagamento na data prevista </t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepção </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Papel higiênico no banheiro da rodoviária!! Nunca tinha </t>
+  </si>
+  <si>
+    <t>Transporte, Local para descanso e cadeiras, Tratamento pelos funcionários efetivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualquer uma que se encaixa a meu desempenho </t>
+  </si>
+  <si>
+    <t>Pintor</t>
+  </si>
+  <si>
+    <t>Escala e folgas, Nada, estava bom</t>
+  </si>
+  <si>
+    <t>O salário é ótimo por apenas dobrar toalhas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">área de limpeza </t>
+  </si>
+  <si>
+    <t>Nao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepcionista de parque </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legal </t>
+  </si>
+  <si>
+    <t>Pós vendas .</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só agradecer pela oportunidade . </t>
+  </si>
+  <si>
+    <t xml:space="preserve">De vendedor </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tudo muito organizado </t>
+  </si>
+  <si>
+    <t>Valor maior da diária, Ajuda de custo para transporte ou alimentação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recreação ou vendas </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seria uma boa ajuda de custo com transporte pois o transporte da empresa não atende os horários de cada equipe. Pela quantidade de trabalho o salário poderia também ser melhor. E se tivesse pelo menos café da manhã disponível nos horários de chegada de todos os funcionários, além do almoço. Já havia trabalhado em temporadas e efetivada com a rh Mendes foi a primeira vez, mas sempre nos trataram bem e com respeito. Agradeço a oportunidade sempre! </t>
+  </si>
+  <si>
+    <t>Gostei muito de trabalhar com  r mendes</t>
+  </si>
+  <si>
+    <t>Monitora de lazer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parabéns a toda equipe </t>
   </si>
 </sst>
 </file>
@@ -786,7 +858,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Q80" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Q94" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="17">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Em qual função você trabalhou na temporada de julho?" id="2"/>
@@ -4235,6 +4307,580 @@
         <v>210</v>
       </c>
     </row>
+    <row r="81" ht="22.5" customHeight="1">
+      <c r="A81" s="5">
+        <v>46245.34378231481</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D81" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G81" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H81" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L81" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="N81" s="6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="82" ht="22.5" customHeight="1">
+      <c r="A82" s="5">
+        <v>46245.34379806713</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D82" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="H82" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q82" s="6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="83" ht="22.5" customHeight="1">
+      <c r="A83" s="5">
+        <v>46245.40759908565</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G83" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H83" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L83" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M83" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q83" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="84" ht="22.5" customHeight="1">
+      <c r="A84" s="5">
+        <v>46245.520437314815</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D84" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H84" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L84" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="P84" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="85" ht="22.5" customHeight="1">
+      <c r="A85" s="5">
+        <v>46246.31773847222</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D85" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="E85" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="H85" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L85" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M85" s="6" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="86" ht="22.5" customHeight="1">
+      <c r="A86" s="5">
+        <v>46246.49371471065</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D86" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="E86" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F86" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G86" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H86" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L86" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M86" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q86" s="6" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="87" ht="22.5" customHeight="1">
+      <c r="A87" s="5">
+        <v>46246.51599082176</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D87" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G87" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="H87" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L87" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M87" s="6" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="88" ht="22.5" customHeight="1">
+      <c r="A88" s="5">
+        <v>46246.82528821759</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D88" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G88" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H88" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J88" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="L88" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="N88" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="O88" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="Q88" s="6" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="89" ht="22.5" customHeight="1">
+      <c r="A89" s="5">
+        <v>46246.85185659722</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H89" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L89" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M89" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q89" s="6" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="90" ht="22.5" customHeight="1">
+      <c r="A90" s="5">
+        <v>46246.863217986116</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D90" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="H90" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L90" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="N90" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="O90" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q90" s="6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="91" ht="22.5" customHeight="1">
+      <c r="A91" s="5">
+        <v>46247.37585841435</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D91" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="H91" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="I91" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L91" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="N91" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O91" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q91" s="6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="92" ht="22.5" customHeight="1">
+      <c r="A92" s="5">
+        <v>46247.60282078704</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D92" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H92" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="I92" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J92" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L92" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="P92" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q92" s="6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="93" ht="22.5" customHeight="1">
+      <c r="A93" s="5">
+        <v>46248.45015741898</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D93" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="H93" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="I93" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="J93" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L93" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="N93" s="6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="94" ht="22.5" customHeight="1">
+      <c r="A94" s="5">
+        <v>46251.38142832176</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D94" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G94" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="H94" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="I94" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="J94" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L94" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M94" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q94" s="6" t="s">
+        <v>234</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>